<commit_message>
remove inferred base mileage and correct Won-dang trip
</commit_message>
<xml_diff>
--- a/backend/app/modules/safety_ledgers/templates/company-vehicle-template.xlsx
+++ b/backend/app/modules/safety_ledgers/templates/company-vehicle-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JSI\besma-safety-ledgers-deploy\backend\app\modules\safety_ledgers\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{88B07AF5-0C9F-4C4C-9793-9509B9B9D903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{7C9E6A9C-AC07-4AA3-810F-17DD9E5313F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{CB2AFB4F-771C-472A-8EBD-756E310E9CF4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{B6893C91-BA84-4112-BBBC-7FC3BE855389}"/>
   </bookViews>
   <sheets>
     <sheet name="7월" sheetId="16" r:id="rId1"/>
@@ -38,7 +38,7 @@
     <author>허승희</author>
   </authors>
   <commentList>
-    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{E2C23149-5D37-4375-85CB-6F3C70B004DE}">
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{93342067-875A-455D-BA81-3E6BB958AF84}">
       <text>
         <r>
           <rPr>
@@ -64,7 +64,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{0F728E4A-9D3A-423A-9118-0D98D7957E0C}">
+    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{934BACA3-2D2B-4868-8BE8-27237CC6CAAD}">
       <text>
         <r>
           <rPr>
@@ -237,7 +237,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{87D18172-C699-47E7-B90E-D0EF89FA6D8A}">
+    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{3ACE5118-F284-4CF1-AFB7-60D3F7B4AB9B}">
       <text>
         <r>
           <rPr>
@@ -337,7 +337,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{5F17F22D-B293-4F13-A5F9-FE686E62C809}">
+    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{13270A86-92BB-4488-B50B-611A9D23B261}">
       <text>
         <r>
           <rPr>
@@ -435,7 +435,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{B69D0E42-BF9E-4D81-860B-B3CA070A8B42}">
+    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{8A1A5ED1-8154-4447-A893-586DBB3D6BE0}">
       <text>
         <r>
           <rPr>
@@ -525,7 +525,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{C442BECD-4FE5-406F-8369-C90058B4C5E6}">
+    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{07A9CB57-370F-4825-866D-24DB04320BB0}">
       <text>
         <r>
           <rPr>
@@ -673,7 +673,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{9B42E0B9-328A-43D9-8526-C229674B7285}">
+    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{538B5BB7-8071-4B9A-A91E-80F5788460B6}">
       <text>
         <r>
           <rPr>
@@ -834,7 +834,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{27DB8417-B15A-43E5-A616-0EA8DF59C2C9}">
+    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{2CB2F630-739C-4EB2-9C23-73739A99A0AA}">
       <text>
         <r>
           <rPr>
@@ -933,7 +933,7 @@
     <author>허승희</author>
   </authors>
   <commentList>
-    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{15959C1F-BA61-45DA-8ACF-47458B6D04DB}">
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{E82A7EF8-31A1-40FF-9F68-9768A7EAF824}">
       <text>
         <r>
           <rPr>
@@ -959,7 +959,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{FE2A7226-4FC7-4252-9927-C0B5D6C40367}">
+    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{63D97036-D15A-4816-8F10-7BBFB51AE28B}">
       <text>
         <r>
           <rPr>
@@ -1132,7 +1132,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{9AC47F28-E98F-4D46-B044-DD386B4DCE2B}">
+    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{AED5AF79-E62B-42C3-B529-E3A43CF267B1}">
       <text>
         <r>
           <rPr>
@@ -1232,7 +1232,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{A63279E2-964D-40AE-BAD1-7B530BAE0C13}">
+    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{5D72941C-84DC-4594-B355-425DA9E6D2CE}">
       <text>
         <r>
           <rPr>
@@ -1330,7 +1330,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{AF2E903D-E13D-4901-8704-03A069AB8E6E}">
+    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{8908EA15-8AF6-427C-BAB0-F8C99B8D990B}">
       <text>
         <r>
           <rPr>
@@ -1420,7 +1420,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{611FE63E-5B95-49D6-8FC2-C18099CA62CF}">
+    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{B7E8C2D7-54A8-464C-B612-3B2296592291}">
       <text>
         <r>
           <rPr>
@@ -1568,7 +1568,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{8F61E9E3-CB32-4689-B857-199148C0D5E9}">
+    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{3D68BEA6-F045-46B2-BA35-163934AF5FB9}">
       <text>
         <r>
           <rPr>
@@ -1729,7 +1729,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{5F7F5104-93FD-493F-9762-6F45C6B56C72}">
+    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{B952A7E4-33E5-4DCD-B4F2-B9774BDBC50E}">
       <text>
         <r>
           <rPr>
@@ -1828,7 +1828,7 @@
     <author>허승희</author>
   </authors>
   <commentList>
-    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{083643E4-2ABB-4F8A-930D-BB5C09201042}">
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{84C09689-06D3-4C3C-BB58-C29D8EAE17FC}">
       <text>
         <r>
           <rPr>
@@ -1854,7 +1854,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{A50853DE-6B6D-4703-A073-5D3F0DD47994}">
+    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{5EACA249-84B9-4EE4-B213-1661F82C8609}">
       <text>
         <r>
           <rPr>
@@ -2027,7 +2027,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{23AA972E-15AD-4BCB-933E-4122ABA295EF}">
+    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{1F4576E5-9DEC-44E7-8142-EEE04C310CAD}">
       <text>
         <r>
           <rPr>
@@ -2127,7 +2127,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{D35AE6AB-7598-493F-B4F4-42CEA1341C7B}">
+    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{0EA6B57D-8F0A-416F-B9A4-4CF5B13B855C}">
       <text>
         <r>
           <rPr>
@@ -2225,7 +2225,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{972D19FF-45BF-4445-A09C-57B09C0BDB49}">
+    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{5B6D0B39-9DFD-48AC-93D0-F70CAF0FC668}">
       <text>
         <r>
           <rPr>
@@ -2315,7 +2315,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{8484DC55-1FF6-4AF0-AF8A-3D37FB248377}">
+    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{A7D2A9B5-6595-4A4B-B76B-DE833B034EDC}">
       <text>
         <r>
           <rPr>
@@ -2463,7 +2463,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{94F462E2-D991-406A-94DD-74505EDD0009}">
+    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{7C585D71-186D-458D-BEE2-286BD1082489}">
       <text>
         <r>
           <rPr>
@@ -2624,7 +2624,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{73159186-5697-40E1-8899-1965BAFEAFC7}">
+    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{6564B96A-BCBA-4349-8646-679AFC221D7C}">
       <text>
         <r>
           <rPr>
@@ -2723,7 +2723,7 @@
     <author>허승희</author>
   </authors>
   <commentList>
-    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{87167485-7593-42D9-9D69-35FD70B5EBA9}">
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{4FAFC940-A094-452D-A36E-933578F65A3E}">
       <text>
         <r>
           <rPr>
@@ -2749,7 +2749,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{21AF5649-77F1-40DF-A6A3-41E17D451617}">
+    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{D4C66204-7263-4D56-8437-CEBA4FC53DB9}">
       <text>
         <r>
           <rPr>
@@ -2922,7 +2922,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{8A107350-9601-49F1-B1BA-D0FDCD208595}">
+    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{0DAF2001-56C6-4CBF-BA7F-8C98D001A678}">
       <text>
         <r>
           <rPr>
@@ -3022,7 +3022,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{CD98427C-6FFA-4D23-A5E3-A39B7C0ABF2A}">
+    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{F6599236-4740-4532-8CE2-57001BBDD186}">
       <text>
         <r>
           <rPr>
@@ -3120,7 +3120,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{BE0E6052-6701-4CD3-8948-039A8328A244}">
+    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{335362C9-2A85-42A8-87C6-B6CA64113742}">
       <text>
         <r>
           <rPr>
@@ -3210,7 +3210,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{76A93796-63B4-4314-83D0-1B364E29473C}">
+    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{800E342C-0C22-4BD5-9011-14FD23F6F1BF}">
       <text>
         <r>
           <rPr>
@@ -3358,7 +3358,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{3E915F44-B587-4B50-8CFE-92D5BE3A1996}">
+    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{DDCC7797-9027-44C7-B735-D0EF049B999A}">
       <text>
         <r>
           <rPr>
@@ -3519,7 +3519,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{683DA72A-E9E4-45D5-A71B-35B831D5186D}">
+    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{873014A0-1913-4386-91BE-C2E9814142FB}">
       <text>
         <r>
           <rPr>
@@ -3618,7 +3618,7 @@
     <author>허승희</author>
   </authors>
   <commentList>
-    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{CAAD54CA-B824-4D28-A5F8-21517D061837}">
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{BCE24386-8BCF-4A1A-8EB9-4C7E0CCE1057}">
       <text>
         <r>
           <rPr>
@@ -3644,7 +3644,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{5729F43C-031C-4571-8F72-972D9EE37041}">
+    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{668477A1-04FB-40CE-9104-A79D8BBE271E}">
       <text>
         <r>
           <rPr>
@@ -3817,7 +3817,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{05B3CA3F-6CDE-43DC-8E2C-EDA3440669D9}">
+    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{27450D01-1638-45C3-993A-4CEBDB1A02F7}">
       <text>
         <r>
           <rPr>
@@ -3917,7 +3917,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{2585D7F2-6C4E-4320-B208-25F4533F9C4B}">
+    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{2F77793D-31FE-4FE1-A84C-CEC97DB86E30}">
       <text>
         <r>
           <rPr>
@@ -4015,7 +4015,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{19B38334-A035-4B79-98BB-3F3B78988AE8}">
+    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{9583C174-D42C-44CE-B890-ADA61F98F403}">
       <text>
         <r>
           <rPr>
@@ -4105,7 +4105,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{393FB187-867E-447F-8DBD-BEC3B31B09D1}">
+    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{226BF609-71DC-4097-99DF-E620DB4040B2}">
       <text>
         <r>
           <rPr>
@@ -4253,7 +4253,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{E2011418-79AE-4FCE-B58E-F35996E76FFE}">
+    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{60E61C84-1033-406A-A7C1-808F94F9C95A}">
       <text>
         <r>
           <rPr>
@@ -4414,7 +4414,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{1928288D-80A1-48C0-B537-154A9D3D091C}">
+    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{381DFF36-DDA1-4BFF-8857-2C22FAD538B3}">
       <text>
         <r>
           <rPr>
@@ -4513,7 +4513,7 @@
     <author>허승희</author>
   </authors>
   <commentList>
-    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{15A1A39C-F915-48AB-8ABE-245865B65A35}">
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{0F201112-9460-418F-8346-B821C64D6416}">
       <text>
         <r>
           <rPr>
@@ -4539,7 +4539,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{0F8F4355-0945-46F1-B039-23F5A469DBC5}">
+    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{95D1538C-D8CF-4338-8B12-0B12F963004B}">
       <text>
         <r>
           <rPr>
@@ -4712,7 +4712,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{C2D3564E-7C4F-4B92-A5F1-CFA67BCF3DC9}">
+    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{8A9BDFE7-BF34-4376-998A-314AABE0E3DC}">
       <text>
         <r>
           <rPr>
@@ -4812,7 +4812,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{82F54A90-ACA3-4481-A662-8C44757E7BB8}">
+    <comment ref="G7" authorId="0" shapeId="0" xr:uid="{93F5CAB4-2697-42E3-ADF3-3FDF8F1C033C}">
       <text>
         <r>
           <rPr>
@@ -4910,7 +4910,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{49B18FA0-0516-4770-9C4B-7428E3F7F2A3}">
+    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{AE6EACF6-4277-4663-828B-C2A2200337E8}">
       <text>
         <r>
           <rPr>
@@ -5000,7 +5000,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{B67EE0D2-CFD7-4172-B8B7-39E145DE6657}">
+    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{DDA6C177-327A-4671-8668-6E2A306FB427}">
       <text>
         <r>
           <rPr>
@@ -5148,7 +5148,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{2EE5AC4A-718C-4680-9723-681A95C49D6D}">
+    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{2B507606-FEC1-4E71-AE9D-0583E82B1CAC}">
       <text>
         <r>
           <rPr>
@@ -5309,7 +5309,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{ABED181D-901B-4048-927D-5346AF3190E1}">
+    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{1D4705F9-24B9-43E5-8291-E7725F981D7E}">
       <text>
         <r>
           <rPr>
@@ -6077,7 +6077,7 @@
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AFBBE59-1982-9BD1-9D1F-9BAA4528393D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB521832-A073-6FDC-48D4-AF6EB8AD940F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6542,7 +6542,7 @@
         <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0DD2A11D-74F2-3AF4-2F9E-A65FE2EAA2AF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{225F0241-C1CB-D1A3-EE22-87E8B9B91181}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6822,7 +6822,7 @@
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2B4CC06B-FD15-43B3-80FD-5C63ACB93773}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9F8FD587-6333-4369-80A4-7FBBE3BD83F9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7287,7 +7287,7 @@
         <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CAEC54C6-F777-4EC7-AAE6-E6C8A903CECD}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5CB2E03E-E237-4A89-9DA2-AA03629788CC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7567,7 +7567,7 @@
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{929CA91A-4ADE-4C99-9433-7C1F58F17C83}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{88F54AEC-25B2-4C72-8C42-84BB97CD1D40}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8032,7 +8032,7 @@
         <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A912FEBF-997D-46BF-A43F-256C79BE4E5C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FEE3E9A7-ED0E-4416-BC81-CD6CFE8FF7CB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8312,7 +8312,7 @@
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C45098E0-14CE-40FD-ACAB-2FC06D8858BB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09B0D424-DFCD-4FC2-99D8-581EC1AD3603}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8777,7 +8777,7 @@
         <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EC076E88-4BE0-4A6F-93D6-B08C579D98BC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8767B58C-DCC4-4374-90B4-0433362F1EA3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9057,7 +9057,7 @@
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB932C3C-15FD-4DF2-AAE6-6D54D446314D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7DEB37F5-9A4A-4414-9603-DD9CBD6A0360}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9522,7 +9522,7 @@
         <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E5E2BF4-E479-4871-A578-F5A88287395C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{66266F40-636A-44BA-A9A3-3A397A7D68F8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9802,7 +9802,7 @@
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{940C7E17-BBF9-4BC0-BCE0-DB469D642C4D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0940FE05-9BF7-407A-B8AD-8AF766B727D7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -10267,7 +10267,7 @@
         <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D43AC0D-3F05-44DD-A593-1748A4498EF5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3A8B5DF2-3E0F-4BE4-B630-B73CDF908194}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -10784,7 +10784,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0725FC66-639F-4C9B-BF2A-DC9BB1F0512C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EDAAC60-15B9-4839-A8E0-B3E38546B798}">
   <dimension ref="A1:L45"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -10909,10 +10909,7 @@
         <v>21</v>
       </c>
       <c r="F7" s="47"/>
-      <c r="G7" s="19" t="e">
-        <f>SUM(#REF!)</f>
-        <v>#REF!</v>
-      </c>
+      <c r="G7" s="19"/>
       <c r="H7" s="23" t="s">
         <v>15</v>
       </c>
@@ -11288,9 +11285,9 @@
       <c r="H41" s="15"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G42" s="22" t="e">
-        <f>SUM(G11:G41,G7)</f>
-        <v>#REF!</v>
+      <c r="G42" s="22">
+        <f>SUM(G11:G41)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -11316,10 +11313,10 @@
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{DE8BE9BD-9F90-4641-81BC-0404529A10E0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{6BDE797B-FEBB-459D-BE21-3E79A8417490}">
       <formula1>"1.출근용,2.퇴근용,3.업무용,4.비업무용(개인),5.출퇴근용(왕복),6.업무용(왕복),7.비업무용(왕복)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{68962381-DC27-4E4F-82A8-C6823B5264A1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{CF5B812B-809C-4DBF-9B34-0C85196F2694}">
       <formula1>"0.회사,1.렌트,2.리스,3.직원,4.타인,5.회사(비),6.리스(비),7.렌트(비)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -11333,7 +11330,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90827B20-CA22-46AC-8967-BE4EA2C64BE0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21C8218F-34C5-4CF9-9BE9-6EBC6A27525A}">
   <dimension ref="A1:L45"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -11458,10 +11455,7 @@
         <v>21</v>
       </c>
       <c r="F7" s="47"/>
-      <c r="G7" s="19" t="e">
-        <f>SUM(#REF!)</f>
-        <v>#REF!</v>
-      </c>
+      <c r="G7" s="19"/>
       <c r="H7" s="23" t="s">
         <v>15</v>
       </c>
@@ -11837,9 +11831,9 @@
       <c r="H41" s="15"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G42" s="22" t="e">
-        <f>SUM(G11:G41,G7)</f>
-        <v>#REF!</v>
+      <c r="G42" s="22">
+        <f>SUM(G11:G41)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -11865,10 +11859,10 @@
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{0A1D84D3-C096-4EB0-99FC-59F278091D18}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{5C08C813-5F0D-4975-A40B-0101DDB229C5}">
       <formula1>"0.회사,1.렌트,2.리스,3.직원,4.타인,5.회사(비),6.리스(비),7.렌트(비)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{1C41738E-8026-4297-9AA4-F7E39F2F7F0D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{6ECC04F8-4009-4C63-965E-2D85BB8F8410}">
       <formula1>"1.출근용,2.퇴근용,3.업무용,4.비업무용(개인),5.출퇴근용(왕복),6.업무용(왕복),7.비업무용(왕복)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -11882,7 +11876,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03D2C1AB-0CF5-48AA-9322-4226F8B1710A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA7FA6BE-9A0A-4240-B5AA-FB430250D19A}">
   <dimension ref="A1:L45"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -12007,10 +12001,7 @@
         <v>21</v>
       </c>
       <c r="F7" s="47"/>
-      <c r="G7" s="19" t="e">
-        <f>SUM(#REF!)</f>
-        <v>#REF!</v>
-      </c>
+      <c r="G7" s="19"/>
       <c r="H7" s="23" t="s">
         <v>15</v>
       </c>
@@ -12386,9 +12377,9 @@
       <c r="H41" s="15"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G42" s="22" t="e">
-        <f>SUM(G11:G41,G7)</f>
-        <v>#REF!</v>
+      <c r="G42" s="22">
+        <f>SUM(G11:G41)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -12414,10 +12405,10 @@
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{8CD1668C-C627-4ADE-BA43-60C2AE112B4F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{67F26B9A-1C8D-4FDE-A4B7-40871C408B91}">
       <formula1>"0.회사,1.렌트,2.리스,3.직원,4.타인,5.회사(비),6.리스(비),7.렌트(비)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{6BC91F3B-501F-4503-87E2-09FF7FF28799}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{613E3230-A62F-4330-B2BC-120294CF615A}">
       <formula1>"1.출근용,2.퇴근용,3.업무용,4.비업무용(개인),5.출퇴근용(왕복),6.업무용(왕복),7.비업무용(왕복)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12431,7 +12422,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{035B9679-1C46-4899-B153-5A0575666863}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D1CF8BD-799C-4582-8D14-9D77046A9DD0}">
   <dimension ref="A1:L45"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -12556,10 +12547,7 @@
         <v>21</v>
       </c>
       <c r="F7" s="47"/>
-      <c r="G7" s="19" t="e">
-        <f>SUM(#REF!)</f>
-        <v>#REF!</v>
-      </c>
+      <c r="G7" s="19"/>
       <c r="H7" s="23" t="s">
         <v>15</v>
       </c>
@@ -12935,9 +12923,9 @@
       <c r="H41" s="15"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G42" s="22" t="e">
-        <f>SUM(G11:G41,G7)</f>
-        <v>#REF!</v>
+      <c r="G42" s="22">
+        <f>SUM(G11:G41)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -12963,10 +12951,10 @@
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{FB59237A-851C-4CD9-8A35-0D88384AD521}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{3C3B9029-44DE-443E-83DE-2C955AC2FCF7}">
       <formula1>"0.회사,1.렌트,2.리스,3.직원,4.타인,5.회사(비),6.리스(비),7.렌트(비)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{1C0F0E1C-5FA8-4B52-9CA5-2C07FD2E4FEE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{D4667D26-8E5D-44FA-9812-6C0BA0ED41E5}">
       <formula1>"1.출근용,2.퇴근용,3.업무용,4.비업무용(개인),5.출퇴근용(왕복),6.업무용(왕복),7.비업무용(왕복)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12980,7 +12968,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53CE8B26-7E9F-4747-87A4-92151E45C83A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECF944FE-F352-4127-AAFD-10FD77121B06}">
   <dimension ref="A1:L45"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -13105,10 +13093,7 @@
         <v>21</v>
       </c>
       <c r="F7" s="47"/>
-      <c r="G7" s="19" t="e">
-        <f>SUM(#REF!)</f>
-        <v>#REF!</v>
-      </c>
+      <c r="G7" s="19"/>
       <c r="H7" s="23" t="s">
         <v>15</v>
       </c>
@@ -13484,9 +13469,9 @@
       <c r="H41" s="15"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G42" s="22" t="e">
-        <f>SUM(G11:G41,G7)</f>
-        <v>#REF!</v>
+      <c r="G42" s="22">
+        <f>SUM(G11:G41)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -13512,10 +13497,10 @@
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{3194DEB3-5025-44EE-AFD1-FBF1B7ED2C60}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{F8EF5814-C6AC-4420-B824-22D033FB72BB}">
       <formula1>"0.회사,1.렌트,2.리스,3.직원,4.타인,5.회사(비),6.리스(비),7.렌트(비)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{A2D511DA-58B9-46E2-BE84-4D3EA48EFC38}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{107BC723-3E3B-4B0C-8CE9-9E061774B5F6}">
       <formula1>"1.출근용,2.퇴근용,3.업무용,4.비업무용(개인),5.출퇴근용(왕복),6.업무용(왕복),7.비업무용(왕복)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -13529,7 +13514,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C64A210E-6ADA-45C0-A340-89C171475BAA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42BA3921-35A5-4E38-A39E-C8D5429DB6A2}">
   <dimension ref="A1:L45"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -13654,10 +13639,7 @@
         <v>21</v>
       </c>
       <c r="F7" s="47"/>
-      <c r="G7" s="19" t="e">
-        <f>SUM(#REF!)</f>
-        <v>#REF!</v>
-      </c>
+      <c r="G7" s="19"/>
       <c r="H7" s="23" t="s">
         <v>15</v>
       </c>
@@ -14033,9 +14015,9 @@
       <c r="H41" s="15"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G42" s="22" t="e">
-        <f>SUM(G11:G41,G7)</f>
-        <v>#REF!</v>
+      <c r="G42" s="22">
+        <f>SUM(G11:G41)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -14061,10 +14043,10 @@
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{84926DC9-B7B2-493A-9776-DB7DD7E01E62}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7" xr:uid="{EAB022D4-FBDC-4429-B418-8B409D0806CD}">
       <formula1>"0.회사,1.렌트,2.리스,3.직원,4.타인,5.회사(비),6.리스(비),7.렌트(비)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{8FBBD658-71A0-4BF9-9536-21CA3BD5D3BA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10:F41" xr:uid="{6B7E3B7F-84B4-42CE-9A4F-9C6302EDA77E}">
       <formula1>"1.출근용,2.퇴근용,3.업무용,4.비업무용(개인),5.출퇴근용(왕복),6.업무용(왕복),7.비업무용(왕복)"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>